<commit_message>
engine updates full suite
</commit_message>
<xml_diff>
--- a/data/team_map.xlsx
+++ b/data/team_map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\durao\Documents\py\abacus-scraper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE75ACE1-9F22-4AFB-9F12-AA0DC7791180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E8A255-FDB9-4E29-853C-357D6D9BF0C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11190" yWindow="0" windowWidth="11460" windowHeight="14410" xr2:uid="{381CAF28-F63E-4E4A-8160-AED9EABCC47A}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11460" windowHeight="14410" xr2:uid="{381CAF28-F63E-4E4A-8160-AED9EABCC47A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="75">
   <si>
     <t>Arizona Cardinals</t>
   </si>
@@ -234,6 +234,33 @@
   </si>
   <si>
     <t>WAS</t>
+  </si>
+  <si>
+    <t>roster_abbrev</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>JAC</t>
+  </si>
+  <si>
+    <t>KC</t>
+  </si>
+  <si>
+    <t>LV</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>SF</t>
+  </si>
+  <si>
+    <t>TB</t>
   </si>
 </sst>
 </file>
@@ -608,277 +635,377 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFEF0B8-9817-4960-8DC0-72003E793C85}">
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>32</v>
       </c>
       <c r="B1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C30" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
     </row>
   </sheetData>

</xml_diff>